<commit_message>
fixes of european football and bugs
</commit_message>
<xml_diff>
--- a/uefa_access_list.xlsx
+++ b/uefa_access_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jens\Documents\fussball-agent-app\FootballAgent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E667C3-5DAF-4375-B70F-F3D681D3129F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A33A2E03-607A-4B00-87FF-DA4392C039C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UCL" sheetId="1" r:id="rId1"/>
@@ -977,17 +977,6 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1002,6 +991,17 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1279,22 +1279,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="4" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -1479,13 +1479,13 @@
       <c r="E14" s="21"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
     </row>
     <row r="17" spans="1:13" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
@@ -1550,13 +1550,13 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
       <c r="H21" t="s">
         <v>147</v>
       </c>
@@ -1577,13 +1577,13 @@
       <c r="B22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="E22" s="29"/>
+      <c r="E22" s="36"/>
     </row>
     <row r="23" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="23">
@@ -1592,13 +1592,13 @@
       <c r="B23" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="34" t="s">
+      <c r="C23" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="E23" s="29"/>
+      <c r="E23" s="36"/>
       <c r="H23" t="s">
         <v>148</v>
       </c>
@@ -1616,13 +1616,13 @@
       <c r="B24" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="D24" s="33" t="s">
+      <c r="D24" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="E24" s="29"/>
+      <c r="E24" s="36"/>
     </row>
     <row r="25" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="23">
@@ -1631,13 +1631,13 @@
       <c r="B25" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="C25" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="D25" s="33" t="s">
+      <c r="D25" s="35" t="s">
         <v>212</v>
       </c>
-      <c r="E25" s="29"/>
+      <c r="E25" s="36"/>
       <c r="H25" t="s">
         <v>149</v>
       </c>
@@ -1655,13 +1655,13 @@
       <c r="B26" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="D26" s="33" t="s">
+      <c r="D26" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E26" s="29"/>
+      <c r="E26" s="36"/>
     </row>
     <row r="27" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="23">
@@ -1670,13 +1670,13 @@
       <c r="B27" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C27" s="34" t="s">
+      <c r="C27" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="E27" s="29"/>
+      <c r="E27" s="36"/>
       <c r="H27" t="s">
         <v>150</v>
       </c>
@@ -1694,13 +1694,13 @@
       <c r="B28" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="35" t="s">
         <v>209</v>
       </c>
-      <c r="E28" s="29"/>
+      <c r="E28" s="36"/>
     </row>
     <row r="29" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="23">
@@ -1709,13 +1709,13 @@
       <c r="B29" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="36"/>
     </row>
     <row r="30" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="23">
@@ -1724,13 +1724,13 @@
       <c r="B30" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="E30" s="29"/>
+      <c r="E30" s="36"/>
     </row>
     <row r="31" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="23">
@@ -1739,13 +1739,13 @@
       <c r="B31" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="E31" s="29"/>
+      <c r="E31" s="36"/>
     </row>
     <row r="32" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="23">
@@ -1754,13 +1754,13 @@
       <c r="B32" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="E32" s="29"/>
+      <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="23">
@@ -1769,13 +1769,13 @@
       <c r="B33" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="35" t="s">
         <v>204</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="36"/>
     </row>
     <row r="34" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="23">
@@ -1784,13 +1784,13 @@
       <c r="B34" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="35" t="s">
         <v>203</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="36"/>
     </row>
     <row r="35" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="23">
@@ -1799,13 +1799,13 @@
       <c r="B35" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="34" t="s">
+      <c r="C35" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="D35" s="33" t="s">
+      <c r="D35" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="E35" s="29"/>
+      <c r="E35" s="36"/>
     </row>
     <row r="36" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="23">
@@ -1814,13 +1814,13 @@
       <c r="B36" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="34" t="s">
+      <c r="C36" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="D36" s="33" t="s">
+      <c r="D36" s="35" t="s">
         <v>201</v>
       </c>
-      <c r="E36" s="29"/>
+      <c r="E36" s="36"/>
     </row>
     <row r="37" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="23">
@@ -1829,13 +1829,13 @@
       <c r="B37" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="C37" s="34" t="s">
+      <c r="C37" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="35" t="s">
         <v>200</v>
       </c>
-      <c r="E37" s="29"/>
+      <c r="E37" s="36"/>
     </row>
     <row r="38" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23">
@@ -1844,13 +1844,13 @@
       <c r="B38" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C38" s="34" t="s">
+      <c r="C38" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="D38" s="33" t="s">
+      <c r="D38" s="35" t="s">
         <v>199</v>
       </c>
-      <c r="E38" s="29"/>
+      <c r="E38" s="36"/>
     </row>
     <row r="39" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="23">
@@ -1859,13 +1859,13 @@
       <c r="B39" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="34" t="s">
+      <c r="C39" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="D39" s="33" t="s">
+      <c r="D39" s="35" t="s">
         <v>198</v>
       </c>
-      <c r="E39" s="29"/>
+      <c r="E39" s="36"/>
     </row>
     <row r="40" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="23">
@@ -1874,13 +1874,13 @@
       <c r="B40" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="34" t="s">
+      <c r="C40" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="D40" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="E40" s="29"/>
+      <c r="E40" s="36"/>
     </row>
     <row r="41" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="23">
@@ -1889,13 +1889,13 @@
       <c r="B41" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="34" t="s">
+      <c r="C41" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="35" t="s">
         <v>196</v>
       </c>
-      <c r="E41" s="29"/>
+      <c r="E41" s="36"/>
     </row>
     <row r="42" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23">
@@ -1904,13 +1904,13 @@
       <c r="B42" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C42" s="34" t="s">
+      <c r="C42" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D42" s="33" t="s">
+      <c r="D42" s="35" t="s">
         <v>195</v>
       </c>
-      <c r="E42" s="29"/>
+      <c r="E42" s="36"/>
     </row>
     <row r="43" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="23">
@@ -1919,13 +1919,13 @@
       <c r="B43" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="34" t="s">
+      <c r="C43" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D43" s="33" t="s">
+      <c r="D43" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="E43" s="29"/>
+      <c r="E43" s="36"/>
     </row>
     <row r="44" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="23">
@@ -1934,13 +1934,13 @@
       <c r="B44" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="C44" s="34" t="s">
+      <c r="C44" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D44" s="33" t="s">
+      <c r="D44" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="E44" s="29"/>
+      <c r="E44" s="36"/>
     </row>
     <row r="45" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="23">
@@ -1949,13 +1949,13 @@
       <c r="B45" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="23">
@@ -1964,13 +1964,13 @@
       <c r="B46" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="C46" s="34" t="s">
+      <c r="C46" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D46" s="33" t="s">
+      <c r="D46" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="E46" s="29"/>
+      <c r="E46" s="36"/>
     </row>
     <row r="47" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="23">
@@ -1979,13 +1979,13 @@
       <c r="B47" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="C47" s="34" t="s">
+      <c r="C47" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D47" s="33" t="s">
+      <c r="D47" s="35" t="s">
         <v>190</v>
       </c>
-      <c r="E47" s="29"/>
+      <c r="E47" s="36"/>
     </row>
     <row r="48" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="23">
@@ -1994,13 +1994,13 @@
       <c r="B48" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="C48" s="34" t="s">
+      <c r="C48" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D48" s="33" t="s">
+      <c r="D48" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="E48" s="29"/>
+      <c r="E48" s="36"/>
     </row>
     <row r="49" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="23">
@@ -2009,13 +2009,13 @@
       <c r="B49" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C49" s="34" t="s">
+      <c r="C49" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D49" s="35" t="s">
         <v>186</v>
       </c>
-      <c r="E49" s="29"/>
+      <c r="E49" s="36"/>
     </row>
     <row r="50" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="23">
@@ -2024,13 +2024,13 @@
       <c r="B50" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="34" t="s">
+      <c r="C50" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D50" s="33" t="s">
+      <c r="D50" s="35" t="s">
         <v>185</v>
       </c>
-      <c r="E50" s="29"/>
+      <c r="E50" s="36"/>
     </row>
     <row r="51" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="23">
@@ -2039,13 +2039,13 @@
       <c r="B51" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="C51" s="34" t="s">
+      <c r="C51" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D51" s="33" t="s">
+      <c r="D51" s="35" t="s">
         <v>184</v>
       </c>
-      <c r="E51" s="29"/>
+      <c r="E51" s="36"/>
     </row>
     <row r="52" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="23">
@@ -2054,13 +2054,13 @@
       <c r="B52" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="C52" s="34" t="s">
+      <c r="C52" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D52" s="33" t="s">
+      <c r="D52" s="35" t="s">
         <v>183</v>
       </c>
-      <c r="E52" s="29"/>
+      <c r="E52" s="36"/>
     </row>
     <row r="53" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="23">
@@ -2069,13 +2069,13 @@
       <c r="B53" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="C53" s="34" t="s">
+      <c r="C53" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="D53" s="29" t="s">
+      <c r="D53" s="36" t="s">
         <v>109</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="36"/>
     </row>
     <row r="54" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="23">
@@ -2084,13 +2084,13 @@
       <c r="B54" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="C54" s="34" t="s">
+      <c r="C54" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D54" s="33" t="s">
+      <c r="D54" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="E54" s="29"/>
+      <c r="E54" s="36"/>
     </row>
     <row r="55" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="23">
@@ -2099,13 +2099,13 @@
       <c r="B55" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="C55" s="34" t="s">
+      <c r="C55" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D55" s="33" t="s">
+      <c r="D55" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="36"/>
     </row>
     <row r="56" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="23">
@@ -2114,13 +2114,13 @@
       <c r="B56" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="C56" s="34" t="s">
+      <c r="C56" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D56" s="33" t="s">
+      <c r="D56" s="35" t="s">
         <v>180</v>
       </c>
-      <c r="E56" s="29"/>
+      <c r="E56" s="36"/>
     </row>
     <row r="57" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="23">
@@ -2129,13 +2129,13 @@
       <c r="B57" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="C57" s="34" t="s">
+      <c r="C57" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D57" s="33" t="s">
+      <c r="D57" s="35" t="s">
         <v>188</v>
       </c>
-      <c r="E57" s="29"/>
+      <c r="E57" s="36"/>
     </row>
     <row r="58" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="23">
@@ -2144,13 +2144,13 @@
       <c r="B58" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C58" s="34" t="s">
+      <c r="C58" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D58" s="33" t="s">
+      <c r="D58" s="35" t="s">
         <v>178</v>
       </c>
-      <c r="E58" s="29"/>
+      <c r="E58" s="36"/>
     </row>
     <row r="59" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="23">
@@ -2159,13 +2159,13 @@
       <c r="B59" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C59" s="34" t="s">
+      <c r="C59" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D59" s="33" t="s">
+      <c r="D59" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="E59" s="29"/>
+      <c r="E59" s="36"/>
     </row>
     <row r="60" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="23">
@@ -2174,13 +2174,13 @@
       <c r="B60" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C60" s="34" t="s">
+      <c r="C60" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D60" s="33" t="s">
+      <c r="D60" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="E60" s="29"/>
+      <c r="E60" s="36"/>
     </row>
     <row r="61" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23">
@@ -2189,13 +2189,13 @@
       <c r="B61" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="C61" s="34" t="s">
+      <c r="C61" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D61" s="33" t="s">
+      <c r="D61" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="E61" s="29"/>
+      <c r="E61" s="36"/>
     </row>
     <row r="62" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="23">
@@ -2204,13 +2204,13 @@
       <c r="B62" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C62" s="34" t="s">
+      <c r="C62" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D62" s="33" t="s">
+      <c r="D62" s="35" t="s">
         <v>174</v>
       </c>
-      <c r="E62" s="29"/>
+      <c r="E62" s="36"/>
     </row>
     <row r="63" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="23">
@@ -2219,13 +2219,13 @@
       <c r="B63" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="C63" s="34" t="s">
+      <c r="C63" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D63" s="33" t="s">
+      <c r="D63" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="E63" s="29"/>
+      <c r="E63" s="36"/>
     </row>
     <row r="64" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="23">
@@ -2234,13 +2234,13 @@
       <c r="B64" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C64" s="34" t="s">
+      <c r="C64" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D64" s="33" t="s">
+      <c r="D64" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="E64" s="29"/>
+      <c r="E64" s="36"/>
     </row>
     <row r="65" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="23">
@@ -2249,13 +2249,13 @@
       <c r="B65" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="C65" s="34" t="s">
+      <c r="C65" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D65" s="33" t="s">
+      <c r="D65" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="E65" s="29"/>
+      <c r="E65" s="36"/>
     </row>
     <row r="66" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="23">
@@ -2264,13 +2264,13 @@
       <c r="B66" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="C66" s="34" t="s">
+      <c r="C66" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D66" s="33" t="s">
+      <c r="D66" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="E66" s="29"/>
+      <c r="E66" s="36"/>
     </row>
     <row r="67" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="23">
@@ -2279,80 +2279,63 @@
       <c r="B67" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="C67" s="34" t="s">
+      <c r="C67" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="D67" s="33" t="s">
+      <c r="D67" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="E67" s="29"/>
+      <c r="E67" s="36"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="30" t="s">
+      <c r="A69" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="B69" s="30"/>
-      <c r="C69" s="30"/>
-      <c r="D69" s="30"/>
-      <c r="E69" s="30"/>
+      <c r="B69" s="34"/>
+      <c r="C69" s="34"/>
+      <c r="D69" s="34"/>
+      <c r="E69" s="34"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="30" t="s">
+      <c r="A70" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="B70" s="30"/>
-      <c r="C70" s="30"/>
-      <c r="D70" s="30"/>
-      <c r="E70" s="30"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="34"/>
+      <c r="D70" s="34"/>
+      <c r="E70" s="34"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="B71" s="30"/>
-      <c r="C71" s="30"/>
-      <c r="D71" s="30"/>
-      <c r="E71" s="30"/>
+      <c r="B71" s="34"/>
+      <c r="C71" s="34"/>
+      <c r="D71" s="34"/>
+      <c r="E71" s="34"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="30" t="s">
+      <c r="A72" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="B72" s="30"/>
-      <c r="C72" s="30"/>
-      <c r="D72" s="30"/>
-      <c r="E72" s="30"/>
+      <c r="B72" s="34"/>
+      <c r="C72" s="34"/>
+      <c r="D72" s="34"/>
+      <c r="E72" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D66:E66"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="D57:E57"/>
@@ -2367,18 +2350,35 @@
     <mergeCell ref="D36:E36"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="D38:E38"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D53:E53"/>
     <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A70:E70"/>
-    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D24:E24"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2400,22 +2400,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="4" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -2535,7 +2535,7 @@
       <c r="C10" s="13">
         <v>2</v>
       </c>
-      <c r="D10" s="36" t="s">
+      <c r="D10" s="31" t="s">
         <v>217</v>
       </c>
       <c r="E10" s="14" t="s">
@@ -2552,7 +2552,7 @@
       <c r="C11" s="15">
         <v>2</v>
       </c>
-      <c r="D11" s="37" t="s">
+      <c r="D11" s="32" t="s">
         <v>218</v>
       </c>
       <c r="E11" s="16" t="s">
@@ -2606,13 +2606,13 @@
       <c r="E14" s="21"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
@@ -2688,13 +2688,13 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
       <c r="H21" t="s">
         <v>148</v>
       </c>
@@ -2712,13 +2712,13 @@
       <c r="B22" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="E22" s="29"/>
+      <c r="E22" s="36"/>
     </row>
     <row r="23" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="23">
@@ -2727,13 +2727,13 @@
       <c r="B23" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="34" t="s">
+      <c r="C23" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="E23" s="29"/>
+      <c r="E23" s="36"/>
       <c r="H23" t="s">
         <v>149</v>
       </c>
@@ -2751,13 +2751,13 @@
       <c r="B24" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D24" s="33" t="s">
+      <c r="D24" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="E24" s="29"/>
+      <c r="E24" s="36"/>
     </row>
     <row r="25" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="23">
@@ -2766,13 +2766,13 @@
       <c r="B25" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="C25" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D25" s="33" t="s">
+      <c r="D25" s="35" t="s">
         <v>212</v>
       </c>
-      <c r="E25" s="29"/>
+      <c r="E25" s="36"/>
       <c r="H25" t="s">
         <v>150</v>
       </c>
@@ -2790,13 +2790,13 @@
       <c r="B26" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D26" s="33" t="s">
+      <c r="D26" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E26" s="29"/>
+      <c r="E26" s="36"/>
     </row>
     <row r="27" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="23">
@@ -2805,13 +2805,13 @@
       <c r="B27" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C27" s="34" t="s">
+      <c r="C27" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="E27" s="29"/>
+      <c r="E27" s="36"/>
       <c r="H27" t="s">
         <v>151</v>
       </c>
@@ -2829,13 +2829,13 @@
       <c r="B28" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="35" t="s">
         <v>209</v>
       </c>
-      <c r="E28" s="29"/>
+      <c r="E28" s="36"/>
     </row>
     <row r="29" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="23">
@@ -2844,13 +2844,13 @@
       <c r="B29" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="36"/>
     </row>
     <row r="30" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="23">
@@ -2859,13 +2859,13 @@
       <c r="B30" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="E30" s="29"/>
+      <c r="E30" s="36"/>
     </row>
     <row r="31" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="23">
@@ -2874,13 +2874,13 @@
       <c r="B31" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="E31" s="29"/>
+      <c r="E31" s="36"/>
     </row>
     <row r="32" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="23">
@@ -2889,13 +2889,13 @@
       <c r="B32" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="E32" s="29"/>
+      <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="23">
@@ -2904,13 +2904,13 @@
       <c r="B33" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="35" t="s">
         <v>204</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="36"/>
     </row>
     <row r="34" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="23">
@@ -2919,13 +2919,13 @@
       <c r="B34" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="35" t="s">
         <v>203</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="36"/>
     </row>
     <row r="35" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="23">
@@ -2934,13 +2934,13 @@
       <c r="B35" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="34" t="s">
+      <c r="C35" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D35" s="33" t="s">
+      <c r="D35" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="E35" s="29"/>
+      <c r="E35" s="36"/>
     </row>
     <row r="36" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="23">
@@ -2949,13 +2949,13 @@
       <c r="B36" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="34" t="s">
+      <c r="C36" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D36" s="33" t="s">
+      <c r="D36" s="35" t="s">
         <v>201</v>
       </c>
-      <c r="E36" s="29"/>
+      <c r="E36" s="36"/>
     </row>
     <row r="37" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="23">
@@ -2964,13 +2964,13 @@
       <c r="B37" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="C37" s="34" t="s">
+      <c r="C37" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="35" t="s">
         <v>200</v>
       </c>
-      <c r="E37" s="29"/>
+      <c r="E37" s="36"/>
     </row>
     <row r="38" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23">
@@ -2979,28 +2979,28 @@
       <c r="B38" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C38" s="34" t="s">
+      <c r="C38" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D38" s="33" t="s">
+      <c r="D38" s="35" t="s">
         <v>199</v>
       </c>
-      <c r="E38" s="29"/>
+      <c r="E38" s="36"/>
     </row>
     <row r="39" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="23">
         <v>27</v>
       </c>
-      <c r="B39" s="35" t="s">
+      <c r="B39" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="34" t="s">
+      <c r="C39" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D39" s="33" t="s">
+      <c r="D39" s="35" t="s">
         <v>198</v>
       </c>
-      <c r="E39" s="29"/>
+      <c r="E39" s="36"/>
     </row>
     <row r="40" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="23">
@@ -3009,13 +3009,13 @@
       <c r="B40" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="34" t="s">
+      <c r="C40" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="D40" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="E40" s="29"/>
+      <c r="E40" s="36"/>
     </row>
     <row r="41" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="23">
@@ -3024,13 +3024,13 @@
       <c r="B41" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="34" t="s">
+      <c r="C41" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="35" t="s">
         <v>196</v>
       </c>
-      <c r="E41" s="29"/>
+      <c r="E41" s="36"/>
     </row>
     <row r="42" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23">
@@ -3039,13 +3039,13 @@
       <c r="B42" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C42" s="34" t="s">
+      <c r="C42" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D42" s="33" t="s">
+      <c r="D42" s="35" t="s">
         <v>195</v>
       </c>
-      <c r="E42" s="29"/>
+      <c r="E42" s="36"/>
     </row>
     <row r="43" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="23">
@@ -3054,13 +3054,13 @@
       <c r="B43" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="34" t="s">
+      <c r="C43" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D43" s="33" t="s">
+      <c r="D43" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="E43" s="29"/>
+      <c r="E43" s="36"/>
     </row>
     <row r="44" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="23">
@@ -3069,13 +3069,13 @@
       <c r="B44" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="C44" s="34" t="s">
+      <c r="C44" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D44" s="33" t="s">
+      <c r="D44" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="E44" s="29"/>
+      <c r="E44" s="36"/>
     </row>
     <row r="45" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="23">
@@ -3084,13 +3084,13 @@
       <c r="B45" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="23">
@@ -3099,13 +3099,13 @@
       <c r="B46" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="C46" s="34" t="s">
+      <c r="C46" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D46" s="33" t="s">
+      <c r="D46" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="E46" s="29"/>
+      <c r="E46" s="36"/>
     </row>
     <row r="47" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="23">
@@ -3114,13 +3114,13 @@
       <c r="B47" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="C47" s="34" t="s">
+      <c r="C47" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D47" s="33" t="s">
+      <c r="D47" s="35" t="s">
         <v>190</v>
       </c>
-      <c r="E47" s="29"/>
+      <c r="E47" s="36"/>
     </row>
     <row r="48" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="23">
@@ -3129,13 +3129,13 @@
       <c r="B48" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="C48" s="34" t="s">
+      <c r="C48" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D48" s="33" t="s">
+      <c r="D48" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="E48" s="29"/>
+      <c r="E48" s="36"/>
     </row>
     <row r="49" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="23">
@@ -3144,13 +3144,13 @@
       <c r="B49" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C49" s="34" t="s">
+      <c r="C49" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D49" s="35" t="s">
         <v>186</v>
       </c>
-      <c r="E49" s="29"/>
+      <c r="E49" s="36"/>
     </row>
     <row r="50" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="23">
@@ -3159,13 +3159,13 @@
       <c r="B50" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="34" t="s">
+      <c r="C50" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D50" s="33" t="s">
+      <c r="D50" s="35" t="s">
         <v>185</v>
       </c>
-      <c r="E50" s="29"/>
+      <c r="E50" s="36"/>
     </row>
     <row r="51" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="23">
@@ -3174,13 +3174,13 @@
       <c r="B51" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="C51" s="34" t="s">
+      <c r="C51" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D51" s="33" t="s">
+      <c r="D51" s="35" t="s">
         <v>184</v>
       </c>
-      <c r="E51" s="29"/>
+      <c r="E51" s="36"/>
     </row>
     <row r="52" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="23">
@@ -3189,13 +3189,13 @@
       <c r="B52" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="C52" s="34" t="s">
+      <c r="C52" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D52" s="33" t="s">
+      <c r="D52" s="35" t="s">
         <v>183</v>
       </c>
-      <c r="E52" s="29"/>
+      <c r="E52" s="36"/>
     </row>
     <row r="53" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="23">
@@ -3204,13 +3204,13 @@
       <c r="B53" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="C53" s="34" t="s">
+      <c r="C53" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="D53" s="33" t="s">
+      <c r="D53" s="35" t="s">
         <v>187</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="36"/>
     </row>
     <row r="54" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="23">
@@ -3219,13 +3219,13 @@
       <c r="B54" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="C54" s="34" t="s">
+      <c r="C54" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="33" t="s">
+      <c r="D54" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="E54" s="29"/>
+      <c r="E54" s="36"/>
     </row>
     <row r="55" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="23">
@@ -3234,13 +3234,13 @@
       <c r="B55" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="C55" s="34" t="s">
+      <c r="C55" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D55" s="33" t="s">
+      <c r="D55" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="36"/>
     </row>
     <row r="56" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="23">
@@ -3249,13 +3249,13 @@
       <c r="B56" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="C56" s="34" t="s">
+      <c r="C56" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D56" s="33" t="s">
+      <c r="D56" s="35" t="s">
         <v>180</v>
       </c>
-      <c r="E56" s="29"/>
+      <c r="E56" s="36"/>
     </row>
     <row r="57" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="23">
@@ -3264,13 +3264,13 @@
       <c r="B57" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="C57" s="34" t="s">
+      <c r="C57" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D57" s="33" t="s">
+      <c r="D57" s="35" t="s">
         <v>179</v>
       </c>
-      <c r="E57" s="29"/>
+      <c r="E57" s="36"/>
     </row>
     <row r="58" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="23">
@@ -3279,13 +3279,13 @@
       <c r="B58" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C58" s="34" t="s">
+      <c r="C58" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D58" s="33" t="s">
+      <c r="D58" s="35" t="s">
         <v>178</v>
       </c>
-      <c r="E58" s="29"/>
+      <c r="E58" s="36"/>
     </row>
     <row r="59" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="23">
@@ -3294,13 +3294,13 @@
       <c r="B59" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C59" s="34" t="s">
+      <c r="C59" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D59" s="33" t="s">
+      <c r="D59" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="E59" s="29"/>
+      <c r="E59" s="36"/>
     </row>
     <row r="60" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="23">
@@ -3309,13 +3309,13 @@
       <c r="B60" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C60" s="34" t="s">
+      <c r="C60" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D60" s="33" t="s">
+      <c r="D60" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="E60" s="29"/>
+      <c r="E60" s="36"/>
     </row>
     <row r="61" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23">
@@ -3324,13 +3324,13 @@
       <c r="B61" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="C61" s="34" t="s">
+      <c r="C61" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D61" s="33" t="s">
+      <c r="D61" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="E61" s="29"/>
+      <c r="E61" s="36"/>
     </row>
     <row r="62" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="23">
@@ -3339,13 +3339,13 @@
       <c r="B62" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C62" s="34" t="s">
+      <c r="C62" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D62" s="33" t="s">
+      <c r="D62" s="35" t="s">
         <v>174</v>
       </c>
-      <c r="E62" s="29"/>
+      <c r="E62" s="36"/>
     </row>
     <row r="63" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="23">
@@ -3354,13 +3354,13 @@
       <c r="B63" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="C63" s="34" t="s">
+      <c r="C63" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D63" s="33" t="s">
+      <c r="D63" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="E63" s="29"/>
+      <c r="E63" s="36"/>
     </row>
     <row r="64" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="23">
@@ -3369,13 +3369,13 @@
       <c r="B64" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C64" s="34" t="s">
+      <c r="C64" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D64" s="33" t="s">
+      <c r="D64" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="E64" s="29"/>
+      <c r="E64" s="36"/>
     </row>
     <row r="65" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="23">
@@ -3384,13 +3384,13 @@
       <c r="B65" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="C65" s="34" t="s">
+      <c r="C65" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D65" s="33" t="s">
+      <c r="D65" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="E65" s="29"/>
+      <c r="E65" s="36"/>
     </row>
     <row r="66" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="23">
@@ -3399,13 +3399,13 @@
       <c r="B66" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="C66" s="34" t="s">
+      <c r="C66" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D66" s="33" t="s">
+      <c r="D66" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="E66" s="29"/>
+      <c r="E66" s="36"/>
     </row>
     <row r="67" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="23">
@@ -3414,49 +3414,84 @@
       <c r="B67" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="C67" s="34" t="s">
+      <c r="C67" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="D67" s="33" t="s">
+      <c r="D67" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="E67" s="29"/>
+      <c r="E67" s="36"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="30"/>
-      <c r="B68" s="30"/>
-      <c r="C68" s="30"/>
-      <c r="D68" s="30"/>
-      <c r="E68" s="30"/>
+      <c r="A68" s="34"/>
+      <c r="B68" s="34"/>
+      <c r="C68" s="34"/>
+      <c r="D68" s="34"/>
+      <c r="E68" s="34"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="30"/>
-      <c r="B69" s="30"/>
-      <c r="C69" s="30"/>
-      <c r="D69" s="30"/>
-      <c r="E69" s="30"/>
+      <c r="A69" s="34"/>
+      <c r="B69" s="34"/>
+      <c r="C69" s="34"/>
+      <c r="D69" s="34"/>
+      <c r="E69" s="34"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="30"/>
-      <c r="B70" s="30"/>
-      <c r="C70" s="30"/>
-      <c r="D70" s="30"/>
-      <c r="E70" s="30"/>
+      <c r="A70" s="34"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="34"/>
+      <c r="D70" s="34"/>
+      <c r="E70" s="34"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="30"/>
-      <c r="B71" s="30"/>
-      <c r="C71" s="30"/>
-      <c r="D71" s="30"/>
-      <c r="E71" s="30"/>
+      <c r="A71" s="34"/>
+      <c r="B71" s="34"/>
+      <c r="C71" s="34"/>
+      <c r="D71" s="34"/>
+      <c r="E71" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A70:E70"/>
-    <mergeCell ref="A71:E71"/>
-    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D57:E57"/>
     <mergeCell ref="D63:E63"/>
     <mergeCell ref="D64:E64"/>
     <mergeCell ref="D65:E65"/>
@@ -3466,46 +3501,11 @@
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="D61:E61"/>
     <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="D67:E67"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3526,22 +3526,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="4" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -3570,7 +3570,7 @@
       <c r="C5" s="3">
         <v>1</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="33" t="s">
         <v>154</v>
       </c>
       <c r="E5" s="4" t="s">
@@ -3655,7 +3655,7 @@
       <c r="C10" s="13">
         <v>1</v>
       </c>
-      <c r="D10" s="36" t="s">
+      <c r="D10" s="31" t="s">
         <v>220</v>
       </c>
       <c r="E10" s="14" t="s">
@@ -3672,7 +3672,7 @@
       <c r="C11" s="15">
         <v>1</v>
       </c>
-      <c r="D11" s="37" t="s">
+      <c r="D11" s="32" t="s">
         <v>221</v>
       </c>
       <c r="E11" s="16" t="s">
@@ -3726,13 +3726,13 @@
       <c r="E14" s="21"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
@@ -3811,13 +3811,13 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="32" t="s">
+      <c r="A22" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
       <c r="H22" t="s">
         <v>149</v>
       </c>
@@ -3835,13 +3835,13 @@
       <c r="B23" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="34" t="s">
+      <c r="C23" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="D23" s="33" t="s">
+      <c r="D23" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="E23" s="29"/>
+      <c r="E23" s="36"/>
     </row>
     <row r="24" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="23">
@@ -3850,13 +3850,13 @@
       <c r="B24" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="D24" s="33" t="s">
+      <c r="D24" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="E24" s="29"/>
+      <c r="E24" s="36"/>
       <c r="H24" t="s">
         <v>150</v>
       </c>
@@ -3874,13 +3874,13 @@
       <c r="B25" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="C25" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="33" t="s">
+      <c r="D25" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="E25" s="29"/>
+      <c r="E25" s="36"/>
     </row>
     <row r="26" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="23">
@@ -3889,13 +3889,13 @@
       <c r="B26" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="D26" s="33" t="s">
+      <c r="D26" s="35" t="s">
         <v>212</v>
       </c>
-      <c r="E26" s="29"/>
+      <c r="E26" s="36"/>
       <c r="H26" t="s">
         <v>151</v>
       </c>
@@ -3913,13 +3913,13 @@
       <c r="B27" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="34" t="s">
+      <c r="C27" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="29"/>
+      <c r="E27" s="36"/>
     </row>
     <row r="28" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="23">
@@ -3928,13 +3928,13 @@
       <c r="B28" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="29" t="s">
         <v>155</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="E28" s="29"/>
+      <c r="E28" s="36"/>
     </row>
     <row r="29" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="23">
@@ -3943,13 +3943,13 @@
       <c r="B29" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="29" t="s">
         <v>155</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="35" t="s">
         <v>209</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="36"/>
     </row>
     <row r="30" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="23">
@@ -3958,13 +3958,13 @@
       <c r="B30" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="E30" s="29"/>
+      <c r="E30" s="36"/>
     </row>
     <row r="31" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="23">
@@ -3973,13 +3973,13 @@
       <c r="B31" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="E31" s="29"/>
+      <c r="E31" s="36"/>
     </row>
     <row r="32" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="23">
@@ -3988,13 +3988,13 @@
       <c r="B32" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="E32" s="29"/>
+      <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="23">
@@ -4003,13 +4003,13 @@
       <c r="B33" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="35" t="s">
         <v>205</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="36"/>
     </row>
     <row r="34" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="23">
@@ -4018,13 +4018,13 @@
       <c r="B34" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="34" t="s">
+      <c r="C34" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="35" t="s">
         <v>204</v>
       </c>
-      <c r="E34" s="29"/>
+      <c r="E34" s="36"/>
     </row>
     <row r="35" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="23">
@@ -4033,13 +4033,13 @@
       <c r="B35" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="34" t="s">
+      <c r="C35" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D35" s="33" t="s">
+      <c r="D35" s="35" t="s">
         <v>203</v>
       </c>
-      <c r="E35" s="29"/>
+      <c r="E35" s="36"/>
     </row>
     <row r="36" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="23">
@@ -4048,13 +4048,13 @@
       <c r="B36" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="34" t="s">
+      <c r="C36" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D36" s="33" t="s">
+      <c r="D36" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="E36" s="29"/>
+      <c r="E36" s="36"/>
     </row>
     <row r="37" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="23">
@@ -4063,13 +4063,13 @@
       <c r="B37" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="34" t="s">
+      <c r="C37" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="35" t="s">
         <v>201</v>
       </c>
-      <c r="E37" s="29"/>
+      <c r="E37" s="36"/>
     </row>
     <row r="38" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23">
@@ -4078,13 +4078,13 @@
       <c r="B38" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="C38" s="34" t="s">
+      <c r="C38" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D38" s="33" t="s">
+      <c r="D38" s="35" t="s">
         <v>200</v>
       </c>
-      <c r="E38" s="29"/>
+      <c r="E38" s="36"/>
     </row>
     <row r="39" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="23">
@@ -4093,28 +4093,28 @@
       <c r="B39" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C39" s="34" t="s">
+      <c r="C39" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="D39" s="33" t="s">
+      <c r="D39" s="35" t="s">
         <v>199</v>
       </c>
-      <c r="E39" s="29"/>
+      <c r="E39" s="36"/>
     </row>
     <row r="40" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="23">
         <v>27</v>
       </c>
-      <c r="B40" s="35" t="s">
+      <c r="B40" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="34" t="s">
+      <c r="C40" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="D40" s="35" t="s">
         <v>198</v>
       </c>
-      <c r="E40" s="29"/>
+      <c r="E40" s="36"/>
     </row>
     <row r="41" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="23">
@@ -4123,13 +4123,13 @@
       <c r="B41" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="34" t="s">
+      <c r="C41" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D41" s="33" t="s">
+      <c r="D41" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="E41" s="29"/>
+      <c r="E41" s="36"/>
     </row>
     <row r="42" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23">
@@ -4138,13 +4138,13 @@
       <c r="B42" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="34" t="s">
+      <c r="C42" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D42" s="33" t="s">
+      <c r="D42" s="35" t="s">
         <v>196</v>
       </c>
-      <c r="E42" s="29"/>
+      <c r="E42" s="36"/>
     </row>
     <row r="43" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="23">
@@ -4153,13 +4153,13 @@
       <c r="B43" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C43" s="34" t="s">
+      <c r="C43" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D43" s="33" t="s">
+      <c r="D43" s="35" t="s">
         <v>195</v>
       </c>
-      <c r="E43" s="29"/>
+      <c r="E43" s="36"/>
     </row>
     <row r="44" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="23">
@@ -4168,13 +4168,13 @@
       <c r="B44" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="34" t="s">
+      <c r="C44" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D44" s="33" t="s">
+      <c r="D44" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="E44" s="29"/>
+      <c r="E44" s="36"/>
     </row>
     <row r="45" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="23">
@@ -4183,13 +4183,13 @@
       <c r="B45" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="23">
@@ -4198,13 +4198,13 @@
       <c r="B46" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="C46" s="34" t="s">
+      <c r="C46" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D46" s="33" t="s">
+      <c r="D46" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="E46" s="29"/>
+      <c r="E46" s="36"/>
     </row>
     <row r="47" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="23">
@@ -4213,13 +4213,13 @@
       <c r="B47" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="C47" s="34" t="s">
+      <c r="C47" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D47" s="33" t="s">
+      <c r="D47" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="E47" s="29"/>
+      <c r="E47" s="36"/>
     </row>
     <row r="48" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="23">
@@ -4228,13 +4228,13 @@
       <c r="B48" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="C48" s="34" t="s">
+      <c r="C48" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D48" s="33" t="s">
+      <c r="D48" s="35" t="s">
         <v>190</v>
       </c>
-      <c r="E48" s="29"/>
+      <c r="E48" s="36"/>
     </row>
     <row r="49" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="23">
@@ -4243,13 +4243,13 @@
       <c r="B49" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="C49" s="34" t="s">
+      <c r="C49" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D49" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="E49" s="29"/>
+      <c r="E49" s="36"/>
     </row>
     <row r="50" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="23">
@@ -4258,13 +4258,13 @@
       <c r="B50" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="34" t="s">
+      <c r="C50" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D50" s="33" t="s">
+      <c r="D50" s="35" t="s">
         <v>186</v>
       </c>
-      <c r="E50" s="29"/>
+      <c r="E50" s="36"/>
     </row>
     <row r="51" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="23">
@@ -4273,13 +4273,13 @@
       <c r="B51" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C51" s="34" t="s">
+      <c r="C51" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D51" s="33" t="s">
+      <c r="D51" s="35" t="s">
         <v>185</v>
       </c>
-      <c r="E51" s="29"/>
+      <c r="E51" s="36"/>
     </row>
     <row r="52" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="23">
@@ -4288,13 +4288,13 @@
       <c r="B52" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="C52" s="34" t="s">
+      <c r="C52" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D52" s="33" t="s">
+      <c r="D52" s="35" t="s">
         <v>184</v>
       </c>
-      <c r="E52" s="29"/>
+      <c r="E52" s="36"/>
     </row>
     <row r="53" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="23">
@@ -4303,13 +4303,13 @@
       <c r="B53" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="C53" s="34" t="s">
+      <c r="C53" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D53" s="33" t="s">
+      <c r="D53" s="35" t="s">
         <v>183</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="36"/>
     </row>
     <row r="54" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="23">
@@ -4318,13 +4318,13 @@
       <c r="B54" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="34" t="s">
+      <c r="C54" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="D54" s="29" t="s">
+      <c r="D54" s="36" t="s">
         <v>109</v>
       </c>
-      <c r="E54" s="29"/>
+      <c r="E54" s="36"/>
     </row>
     <row r="55" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="23">
@@ -4333,13 +4333,13 @@
       <c r="B55" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="C55" s="34" t="s">
+      <c r="C55" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D55" s="33" t="s">
+      <c r="D55" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="36"/>
     </row>
     <row r="56" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="23">
@@ -4348,13 +4348,13 @@
       <c r="B56" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="34" t="s">
+      <c r="C56" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D56" s="33" t="s">
+      <c r="D56" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="E56" s="29"/>
+      <c r="E56" s="36"/>
     </row>
     <row r="57" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="23">
@@ -4363,13 +4363,13 @@
       <c r="B57" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="C57" s="34" t="s">
+      <c r="C57" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D57" s="33" t="s">
+      <c r="D57" s="35" t="s">
         <v>180</v>
       </c>
-      <c r="E57" s="29"/>
+      <c r="E57" s="36"/>
     </row>
     <row r="58" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="23">
@@ -4378,13 +4378,13 @@
       <c r="B58" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="C58" s="34" t="s">
+      <c r="C58" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D58" s="33" t="s">
+      <c r="D58" s="35" t="s">
         <v>179</v>
       </c>
-      <c r="E58" s="29"/>
+      <c r="E58" s="36"/>
     </row>
     <row r="59" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="23">
@@ -4393,13 +4393,13 @@
       <c r="B59" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C59" s="34" t="s">
+      <c r="C59" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D59" s="33" t="s">
+      <c r="D59" s="35" t="s">
         <v>178</v>
       </c>
-      <c r="E59" s="29"/>
+      <c r="E59" s="36"/>
     </row>
     <row r="60" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="23">
@@ -4408,13 +4408,13 @@
       <c r="B60" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C60" s="34" t="s">
+      <c r="C60" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D60" s="33" t="s">
+      <c r="D60" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="E60" s="29"/>
+      <c r="E60" s="36"/>
     </row>
     <row r="61" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23">
@@ -4423,13 +4423,13 @@
       <c r="B61" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C61" s="34" t="s">
+      <c r="C61" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D61" s="33" t="s">
+      <c r="D61" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="E61" s="29"/>
+      <c r="E61" s="36"/>
     </row>
     <row r="62" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="23">
@@ -4438,13 +4438,13 @@
       <c r="B62" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="C62" s="34" t="s">
+      <c r="C62" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D62" s="33" t="s">
+      <c r="D62" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="E62" s="29"/>
+      <c r="E62" s="36"/>
     </row>
     <row r="63" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="23">
@@ -4453,13 +4453,13 @@
       <c r="B63" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C63" s="34" t="s">
+      <c r="C63" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D63" s="33" t="s">
+      <c r="D63" s="35" t="s">
         <v>174</v>
       </c>
-      <c r="E63" s="29"/>
+      <c r="E63" s="36"/>
     </row>
     <row r="64" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="23">
@@ -4468,13 +4468,13 @@
       <c r="B64" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="C64" s="34" t="s">
+      <c r="C64" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D64" s="33" t="s">
+      <c r="D64" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="E64" s="29"/>
+      <c r="E64" s="36"/>
     </row>
     <row r="65" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="23">
@@ -4483,13 +4483,13 @@
       <c r="B65" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C65" s="34" t="s">
+      <c r="C65" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D65" s="33" t="s">
+      <c r="D65" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="E65" s="29"/>
+      <c r="E65" s="36"/>
     </row>
     <row r="66" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="23">
@@ -4498,13 +4498,13 @@
       <c r="B66" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="C66" s="34" t="s">
+      <c r="C66" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D66" s="33" t="s">
+      <c r="D66" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="E66" s="29"/>
+      <c r="E66" s="36"/>
     </row>
     <row r="67" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="23">
@@ -4513,13 +4513,13 @@
       <c r="B67" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="C67" s="34" t="s">
+      <c r="C67" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D67" s="33" t="s">
+      <c r="D67" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="E67" s="29"/>
+      <c r="E67" s="36"/>
     </row>
     <row r="68" spans="1:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="23">
@@ -4528,66 +4528,66 @@
       <c r="B68" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="C68" s="34" t="s">
+      <c r="C68" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="D68" s="33" t="s">
+      <c r="D68" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="E68" s="29"/>
+      <c r="E68" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D68:E68"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>